<commit_message>
Name change and  clustering
</commit_message>
<xml_diff>
--- a/Input/FantaSPL_V2.3.xlsx
+++ b/Input/FantaSPL_V2.3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Local_Docs\Admin\Other\Kit\SPL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0FED7B2-5C3A-48DB-BF9B-73BBA4D962B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F4E1AFA-F941-4F23-9A7F-4B7E86CDDF7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{05F018D4-855F-4570-8D15-9B4DD092A228}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{05F018D4-855F-4570-8D15-9B4DD092A228}"/>
   </bookViews>
   <sheets>
     <sheet name="Parameters" sheetId="11" r:id="rId1"/>
@@ -21,7 +21,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Players!$A$1:$E$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Points!$A$1:$I$422</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Points!$A$1:$J$440</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1271" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1271" uniqueCount="110">
   <si>
     <t>Parameter</t>
   </si>
@@ -218,9 +218,6 @@
   </si>
   <si>
     <t>Dario (Francesco)</t>
-  </si>
-  <si>
-    <t>Daniele (Francesco)</t>
   </si>
   <si>
     <t>Ale (Mazzu)</t>
@@ -996,7 +993,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="24" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B4" s="25">
         <v>0</v>
@@ -1108,7 +1105,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="24" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B12" s="25">
         <v>10</v>
@@ -1550,7 +1547,7 @@
         <v>9</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
@@ -1611,7 +1608,7 @@
         <v>0</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
@@ -1909,7 +1906,7 @@
         <v>44938</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>30</v>
@@ -2228,7 +2225,7 @@
         <v>44945</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C25" s="9" t="s">
         <v>30</v>
@@ -2542,7 +2539,7 @@
         <v>0</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.35">
@@ -2927,7 +2924,7 @@
         <v>44952</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C49" s="9" t="s">
         <v>22</v>
@@ -2985,7 +2982,7 @@
         <v>44952</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C51" s="9" t="s">
         <v>22</v>
@@ -3072,7 +3069,7 @@
         <v>44959</v>
       </c>
       <c r="B54" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C54" s="9" t="s">
         <v>22</v>
@@ -3130,7 +3127,7 @@
         <v>44959</v>
       </c>
       <c r="B56" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C56" s="9" t="s">
         <v>22</v>
@@ -3420,7 +3417,7 @@
         <v>44959</v>
       </c>
       <c r="B66" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C66" s="9" t="s">
         <v>30</v>
@@ -3710,7 +3707,7 @@
         <v>44966</v>
       </c>
       <c r="B76" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C76" s="9" t="s">
         <v>30</v>
@@ -3971,7 +3968,7 @@
         <v>44980</v>
       </c>
       <c r="B85" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C85" s="9" t="s">
         <v>22</v>
@@ -4145,7 +4142,7 @@
         <v>44980</v>
       </c>
       <c r="B91" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C91" s="9" t="s">
         <v>30</v>
@@ -4725,7 +4722,7 @@
         <v>44987</v>
       </c>
       <c r="B111" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C111" s="9" t="s">
         <v>22</v>
@@ -4899,7 +4896,7 @@
         <v>44994</v>
       </c>
       <c r="B117" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C117" s="9" t="s">
         <v>30</v>
@@ -5015,7 +5012,7 @@
         <v>44994</v>
       </c>
       <c r="B121" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C121" s="9" t="s">
         <v>22</v>
@@ -5044,7 +5041,7 @@
         <v>44994</v>
       </c>
       <c r="B122" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C122" s="9" t="s">
         <v>22</v>
@@ -5073,7 +5070,7 @@
         <v>44994</v>
       </c>
       <c r="B123" s="8" t="s">
-        <v>58</v>
+        <v>95</v>
       </c>
       <c r="C123" s="9" t="s">
         <v>22</v>
@@ -5189,7 +5186,7 @@
         <v>45001</v>
       </c>
       <c r="B127" s="8" t="s">
-        <v>58</v>
+        <v>95</v>
       </c>
       <c r="C127" s="9" t="s">
         <v>22</v>
@@ -5334,7 +5331,7 @@
         <v>45001</v>
       </c>
       <c r="B132" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C132" s="9" t="s">
         <v>22</v>
@@ -5392,7 +5389,7 @@
         <v>45001</v>
       </c>
       <c r="B134" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C134" s="9" t="s">
         <v>30</v>
@@ -5769,7 +5766,7 @@
         <v>45008</v>
       </c>
       <c r="B147" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C147" s="9" t="s">
         <v>30</v>
@@ -5798,7 +5795,7 @@
         <v>45008</v>
       </c>
       <c r="B148" s="8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C148" s="9" t="s">
         <v>30</v>
@@ -5943,7 +5940,7 @@
         <v>45008</v>
       </c>
       <c r="B153" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C153" s="9" t="s">
         <v>30</v>
@@ -6233,7 +6230,7 @@
         <v>45015</v>
       </c>
       <c r="B163" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C163" s="9" t="s">
         <v>30</v>
@@ -6262,7 +6259,7 @@
         <v>45015</v>
       </c>
       <c r="B164" s="8" t="s">
-        <v>58</v>
+        <v>95</v>
       </c>
       <c r="C164" s="9" t="s">
         <v>30</v>
@@ -6291,7 +6288,7 @@
         <v>45015</v>
       </c>
       <c r="B165" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C165" s="9" t="s">
         <v>30</v>
@@ -6320,7 +6317,7 @@
         <v>45015</v>
       </c>
       <c r="B166" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C166" s="9" t="s">
         <v>30</v>
@@ -6755,7 +6752,7 @@
         <v>45022</v>
       </c>
       <c r="B181" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C181" s="9" t="s">
         <v>22</v>
@@ -6784,7 +6781,7 @@
         <v>45030</v>
       </c>
       <c r="B182" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C182" s="9" t="s">
         <v>30</v>
@@ -6958,7 +6955,7 @@
         <v>45030</v>
       </c>
       <c r="B188" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C188" s="9" t="s">
         <v>30</v>
@@ -7103,7 +7100,7 @@
         <v>45030</v>
       </c>
       <c r="B193" s="8" t="s">
-        <v>58</v>
+        <v>95</v>
       </c>
       <c r="C193" s="9" t="s">
         <v>22</v>
@@ -7219,7 +7216,7 @@
         <v>45030</v>
       </c>
       <c r="B197" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C197" s="9" t="s">
         <v>22</v>
@@ -7306,7 +7303,7 @@
         <v>45030</v>
       </c>
       <c r="B200" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C200" s="9" t="s">
         <v>22</v>
@@ -7335,7 +7332,7 @@
         <v>45030</v>
       </c>
       <c r="B201" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C201" s="9" t="s">
         <v>22</v>
@@ -7480,7 +7477,7 @@
         <v>45050</v>
       </c>
       <c r="B206" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C206" s="9" t="s">
         <v>22</v>
@@ -7567,7 +7564,7 @@
         <v>45050</v>
       </c>
       <c r="B209" s="10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C209" s="9" t="s">
         <v>22</v>
@@ -7799,7 +7796,7 @@
         <v>45050</v>
       </c>
       <c r="B217" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C217" s="9" t="s">
         <v>30</v>
@@ -7828,7 +7825,7 @@
         <v>45050</v>
       </c>
       <c r="B218" s="8" t="s">
-        <v>58</v>
+        <v>95</v>
       </c>
       <c r="C218" s="9" t="s">
         <v>30</v>
@@ -8002,7 +7999,7 @@
         <v>45057</v>
       </c>
       <c r="B224" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C224" s="9" t="s">
         <v>30</v>
@@ -8031,7 +8028,7 @@
         <v>45057</v>
       </c>
       <c r="B225" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C225" s="9" t="s">
         <v>30</v>
@@ -8147,7 +8144,7 @@
         <v>45057</v>
       </c>
       <c r="B229" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C229" s="9" t="s">
         <v>22</v>
@@ -8234,7 +8231,7 @@
         <v>45057</v>
       </c>
       <c r="B232" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C232" s="9" t="s">
         <v>22</v>
@@ -8263,7 +8260,7 @@
         <v>45057</v>
       </c>
       <c r="B233" s="8" t="s">
-        <v>58</v>
+        <v>95</v>
       </c>
       <c r="C233" s="9" t="s">
         <v>22</v>
@@ -8408,7 +8405,7 @@
         <v>45064</v>
       </c>
       <c r="B238" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C238" s="9" t="s">
         <v>22</v>
@@ -8437,7 +8434,7 @@
         <v>45064</v>
       </c>
       <c r="B239" s="8" t="s">
-        <v>58</v>
+        <v>95</v>
       </c>
       <c r="C239" s="9" t="s">
         <v>22</v>
@@ -8466,7 +8463,7 @@
         <v>45064</v>
       </c>
       <c r="B240" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C240" s="9" t="s">
         <v>22</v>
@@ -8495,7 +8492,7 @@
         <v>45064</v>
       </c>
       <c r="B241" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C241" s="9" t="s">
         <v>22</v>
@@ -8582,7 +8579,7 @@
         <v>45064</v>
       </c>
       <c r="B244" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C244" s="9" t="s">
         <v>30</v>
@@ -8611,7 +8608,7 @@
         <v>45064</v>
       </c>
       <c r="B245" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C245" s="9" t="s">
         <v>30</v>
@@ -8814,7 +8811,7 @@
         <v>45071</v>
       </c>
       <c r="B252" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C252" s="9" t="s">
         <v>22</v>
@@ -8988,7 +8985,7 @@
         <v>45071</v>
       </c>
       <c r="B258" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C258" s="9" t="s">
         <v>30</v>
@@ -9017,7 +9014,7 @@
         <v>45071</v>
       </c>
       <c r="B259" s="8" t="s">
-        <v>58</v>
+        <v>95</v>
       </c>
       <c r="C259" s="9" t="s">
         <v>30</v>
@@ -9075,7 +9072,7 @@
         <v>45071</v>
       </c>
       <c r="B261" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C261" s="9" t="s">
         <v>30</v>
@@ -9394,7 +9391,7 @@
         <v>45078</v>
       </c>
       <c r="B272" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C272" s="9" t="s">
         <v>30</v>
@@ -9452,7 +9449,7 @@
         <v>45078</v>
       </c>
       <c r="B274" s="8" t="s">
-        <v>58</v>
+        <v>95</v>
       </c>
       <c r="C274" s="9" t="s">
         <v>30</v>
@@ -9481,7 +9478,7 @@
         <v>45078</v>
       </c>
       <c r="B275" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C275" s="9" t="s">
         <v>30</v>
@@ -9539,7 +9536,7 @@
         <v>45078</v>
       </c>
       <c r="B277" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C277" s="9" t="s">
         <v>30</v>
@@ -9800,7 +9797,7 @@
         <v>45085</v>
       </c>
       <c r="B286" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C286" s="9" t="s">
         <v>22</v>
@@ -9829,7 +9826,7 @@
         <v>45085</v>
       </c>
       <c r="B287" s="8" t="s">
-        <v>58</v>
+        <v>95</v>
       </c>
       <c r="C287" s="9" t="s">
         <v>22</v>
@@ -9858,7 +9855,7 @@
         <v>45085</v>
       </c>
       <c r="B288" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C288" s="9" t="s">
         <v>22</v>
@@ -9887,7 +9884,7 @@
         <v>45085</v>
       </c>
       <c r="B289" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C289" s="9" t="s">
         <v>22</v>
@@ -9945,7 +9942,7 @@
         <v>45085</v>
       </c>
       <c r="B291" s="8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C291" s="9" t="s">
         <v>22</v>
@@ -10061,7 +10058,7 @@
         <v>45092</v>
       </c>
       <c r="B295" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C295" s="9" t="s">
         <v>22</v>
@@ -10119,7 +10116,7 @@
         <v>45092</v>
       </c>
       <c r="B297" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C297" s="9" t="s">
         <v>22</v>
@@ -10148,7 +10145,7 @@
         <v>45092</v>
       </c>
       <c r="B298" s="8" t="s">
-        <v>58</v>
+        <v>95</v>
       </c>
       <c r="C298" s="9" t="s">
         <v>22</v>
@@ -10206,7 +10203,7 @@
         <v>45092</v>
       </c>
       <c r="B300" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C300" s="9" t="s">
         <v>30</v>
@@ -10264,7 +10261,7 @@
         <v>45092</v>
       </c>
       <c r="B302" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C302" s="9" t="s">
         <v>30</v>
@@ -10409,7 +10406,7 @@
         <v>45092</v>
       </c>
       <c r="B307" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C307" s="9" t="s">
         <v>30</v>
@@ -10496,7 +10493,7 @@
         <v>45099</v>
       </c>
       <c r="B310" s="8" t="s">
-        <v>58</v>
+        <v>95</v>
       </c>
       <c r="C310" s="9" t="s">
         <v>30</v>
@@ -10525,7 +10522,7 @@
         <v>45099</v>
       </c>
       <c r="B311" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C311" s="9" t="s">
         <v>30</v>
@@ -10583,7 +10580,7 @@
         <v>45099</v>
       </c>
       <c r="B313" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C313" s="9" t="s">
         <v>30</v>
@@ -10612,7 +10609,7 @@
         <v>45099</v>
       </c>
       <c r="B314" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C314" s="9" t="s">
         <v>30</v>
@@ -10786,7 +10783,7 @@
         <v>45099</v>
       </c>
       <c r="B320" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C320" s="9" t="s">
         <v>22</v>
@@ -10815,7 +10812,7 @@
         <v>45099</v>
       </c>
       <c r="B321" s="8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C321" s="9" t="s">
         <v>22</v>
@@ -11076,7 +11073,7 @@
         <v>45106</v>
       </c>
       <c r="B330" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C330" s="9" t="s">
         <v>30</v>
@@ -11105,7 +11102,7 @@
         <v>45106</v>
       </c>
       <c r="B331" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C331" s="9" t="s">
         <v>30</v>
@@ -11163,7 +11160,7 @@
         <v>45106</v>
       </c>
       <c r="B333" s="8" t="s">
-        <v>58</v>
+        <v>95</v>
       </c>
       <c r="C333" s="9" t="s">
         <v>22</v>
@@ -11192,7 +11189,7 @@
         <v>45106</v>
       </c>
       <c r="B334" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C334" s="9" t="s">
         <v>22</v>
@@ -11221,7 +11218,7 @@
         <v>45106</v>
       </c>
       <c r="B335" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C335" s="9" t="s">
         <v>22</v>
@@ -11279,7 +11276,7 @@
         <v>45106</v>
       </c>
       <c r="B337" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C337" s="9" t="s">
         <v>22</v>
@@ -11395,7 +11392,7 @@
         <v>45113</v>
       </c>
       <c r="B341" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C341" s="9" t="s">
         <v>30</v>
@@ -11482,7 +11479,7 @@
         <v>45113</v>
       </c>
       <c r="B344" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C344" s="9" t="s">
         <v>30</v>
@@ -11511,7 +11508,7 @@
         <v>45113</v>
       </c>
       <c r="B345" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C345" s="9" t="s">
         <v>30</v>
@@ -11540,7 +11537,7 @@
         <v>45113</v>
       </c>
       <c r="B346" s="8" t="s">
-        <v>58</v>
+        <v>95</v>
       </c>
       <c r="C346" s="9" t="s">
         <v>30</v>
@@ -11743,7 +11740,7 @@
         <v>45113</v>
       </c>
       <c r="B353" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C353" s="9" t="s">
         <v>22</v>
@@ -11772,7 +11769,7 @@
         <v>45114</v>
       </c>
       <c r="B354" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C354" s="9" t="s">
         <v>22</v>
@@ -11859,7 +11856,7 @@
         <v>45114</v>
       </c>
       <c r="B357" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C357" s="9" t="s">
         <v>22</v>
@@ -11946,7 +11943,7 @@
         <v>45114</v>
       </c>
       <c r="B360" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C360" s="9" t="s">
         <v>22</v>
@@ -11975,7 +11972,7 @@
         <v>45114</v>
       </c>
       <c r="B361" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C361" s="9" t="s">
         <v>30</v>
@@ -12033,7 +12030,7 @@
         <v>45114</v>
       </c>
       <c r="B363" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C363" s="9" t="s">
         <v>30</v>
@@ -12062,7 +12059,7 @@
         <v>45114</v>
       </c>
       <c r="B364" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C364" s="9" t="s">
         <v>30</v>
@@ -12178,7 +12175,7 @@
         <v>45115</v>
       </c>
       <c r="B368" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C368" s="9" t="s">
         <v>30</v>
@@ -12207,7 +12204,7 @@
         <v>45115</v>
       </c>
       <c r="B369" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C369" s="9" t="s">
         <v>30</v>
@@ -12265,7 +12262,7 @@
         <v>45115</v>
       </c>
       <c r="B371" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C371" s="9" t="s">
         <v>30</v>
@@ -12294,7 +12291,7 @@
         <v>45115</v>
       </c>
       <c r="B372" s="8" t="s">
-        <v>58</v>
+        <v>95</v>
       </c>
       <c r="C372" s="9" t="s">
         <v>22</v>
@@ -12323,7 +12320,7 @@
         <v>45115</v>
       </c>
       <c r="B373" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C373" s="9" t="s">
         <v>22</v>
@@ -12410,7 +12407,7 @@
         <v>45115</v>
       </c>
       <c r="B376" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C376" s="9" t="s">
         <v>22</v>
@@ -12439,7 +12436,7 @@
         <v>45116</v>
       </c>
       <c r="B377" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C377" s="9" t="s">
         <v>30</v>
@@ -12497,7 +12494,7 @@
         <v>45116</v>
       </c>
       <c r="B379" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C379" s="9" t="s">
         <v>30</v>
@@ -12555,7 +12552,7 @@
         <v>45116</v>
       </c>
       <c r="B381" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C381" s="9" t="s">
         <v>30</v>
@@ -12584,7 +12581,7 @@
         <v>45116</v>
       </c>
       <c r="B382" s="8" t="s">
-        <v>58</v>
+        <v>95</v>
       </c>
       <c r="C382" s="9" t="s">
         <v>30</v>
@@ -12642,7 +12639,7 @@
         <v>45116</v>
       </c>
       <c r="B384" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C384" s="9" t="s">
         <v>22</v>
@@ -12700,7 +12697,7 @@
         <v>45116</v>
       </c>
       <c r="B386" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C386" s="9" t="s">
         <v>22</v>
@@ -12787,7 +12784,7 @@
         <v>45116</v>
       </c>
       <c r="B389" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C389" s="9" t="s">
         <v>22</v>
@@ -12874,7 +12871,7 @@
         <v>45117</v>
       </c>
       <c r="B392" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C392" s="9" t="s">
         <v>30</v>
@@ -12903,7 +12900,7 @@
         <v>45117</v>
       </c>
       <c r="B393" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C393" s="9" t="s">
         <v>30</v>
@@ -13019,7 +13016,7 @@
         <v>45117</v>
       </c>
       <c r="B397" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C397" s="9" t="s">
         <v>22</v>
@@ -13048,7 +13045,7 @@
         <v>45117</v>
       </c>
       <c r="B398" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C398" s="9" t="s">
         <v>22</v>
@@ -13077,7 +13074,7 @@
         <v>45117</v>
       </c>
       <c r="B399" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C399" s="9" t="s">
         <v>22</v>
@@ -13135,7 +13132,7 @@
         <v>45118</v>
       </c>
       <c r="B401" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C401" s="9" t="s">
         <v>30</v>
@@ -13193,7 +13190,7 @@
         <v>45118</v>
       </c>
       <c r="B403" s="8" t="s">
-        <v>58</v>
+        <v>95</v>
       </c>
       <c r="C403" s="9" t="s">
         <v>30</v>
@@ -13251,7 +13248,7 @@
         <v>45118</v>
       </c>
       <c r="B405" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C405" s="9" t="s">
         <v>30</v>
@@ -13309,7 +13306,7 @@
         <v>45118</v>
       </c>
       <c r="B407" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C407" s="9" t="s">
         <v>22</v>
@@ -13396,7 +13393,7 @@
         <v>45118</v>
       </c>
       <c r="B410" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C410" s="9" t="s">
         <v>22</v>
@@ -13483,7 +13480,7 @@
         <v>45118</v>
       </c>
       <c r="B413" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C413" s="9" t="s">
         <v>22</v>
@@ -13512,7 +13509,7 @@
         <v>45119</v>
       </c>
       <c r="B414" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C414" s="9" t="s">
         <v>30</v>
@@ -13570,7 +13567,7 @@
         <v>45119</v>
       </c>
       <c r="B416" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C416" s="9" t="s">
         <v>30</v>
@@ -13599,7 +13596,7 @@
         <v>45119</v>
       </c>
       <c r="B417" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C417" s="9" t="s">
         <v>30</v>
@@ -13657,7 +13654,7 @@
         <v>45119</v>
       </c>
       <c r="B419" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C419" s="9" t="s">
         <v>22</v>
@@ -13715,7 +13712,7 @@
         <v>45119</v>
       </c>
       <c r="B421" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C421" s="9" t="s">
         <v>22</v>
@@ -13744,7 +13741,7 @@
         <v>45119</v>
       </c>
       <c r="B422" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C422" s="9" t="s">
         <v>22</v>
@@ -13773,7 +13770,7 @@
         <v>45170</v>
       </c>
       <c r="B423" s="29" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C423" s="30" t="s">
         <v>30</v>
@@ -13797,7 +13794,7 @@
         <v>0</v>
       </c>
       <c r="J423" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="424" spans="1:10" x14ac:dyDescent="0.35">
@@ -13834,7 +13831,7 @@
         <v>45170</v>
       </c>
       <c r="B425" s="29" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C425" s="30" t="s">
         <v>30</v>
@@ -13863,7 +13860,7 @@
         <v>45170</v>
       </c>
       <c r="B426" s="29" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C426" s="30" t="s">
         <v>30</v>
@@ -13921,7 +13918,7 @@
         <v>45170</v>
       </c>
       <c r="B428" s="29" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C428" s="30" t="s">
         <v>22</v>
@@ -13979,7 +13976,7 @@
         <v>45170</v>
       </c>
       <c r="B430" s="29" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C430" s="30" t="s">
         <v>22</v>
@@ -14008,7 +14005,7 @@
         <v>45170</v>
       </c>
       <c r="B431" s="29" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C431" s="30" t="s">
         <v>22</v>
@@ -14037,7 +14034,7 @@
         <v>45179</v>
       </c>
       <c r="B432" s="29" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C432" s="30" t="s">
         <v>30</v>
@@ -14061,7 +14058,7 @@
         <v>0</v>
       </c>
       <c r="J432" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="433" spans="1:10" x14ac:dyDescent="0.35">
@@ -14098,7 +14095,7 @@
         <v>45179</v>
       </c>
       <c r="B434" s="29" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C434" s="30" t="s">
         <v>30</v>
@@ -14122,7 +14119,7 @@
         <v>0</v>
       </c>
       <c r="J434" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="435" spans="1:10" x14ac:dyDescent="0.35">
@@ -14130,7 +14127,7 @@
         <v>45179</v>
       </c>
       <c r="B435" s="29" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C435" s="30" t="s">
         <v>30</v>
@@ -14188,7 +14185,7 @@
         <v>45179</v>
       </c>
       <c r="B437" s="29" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C437" s="30" t="s">
         <v>22</v>
@@ -14246,7 +14243,7 @@
         <v>45179</v>
       </c>
       <c r="B439" s="29" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C439" s="30" t="s">
         <v>22</v>
@@ -14275,7 +14272,7 @@
         <v>45179</v>
       </c>
       <c r="B440" s="29" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C440" s="30" t="s">
         <v>22</v>
@@ -14300,6 +14297,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:J440" xr:uid="{F55E8A24-46F9-4225-A2C2-A9164F13364A}"/>
   <conditionalFormatting sqref="C2:C440">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"Scuri"</formula>
@@ -14352,36 +14350,36 @@
         <v>16</v>
       </c>
       <c r="B1" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="D1" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="E1" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="E1" s="16" t="s">
+      <c r="F1" s="16" t="s">
         <v>85</v>
-      </c>
-      <c r="F1" s="16" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C2" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D2" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="E2" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E2" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F2" s="19" t="s">
         <v>29</v>
@@ -14389,19 +14387,19 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="19" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C3" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="D3" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="D3" s="21" t="s">
-        <v>91</v>
-      </c>
       <c r="E3" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F3" s="19" t="s">
         <v>26</v>
@@ -14409,19 +14407,19 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C4" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="D4" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="D4" s="21" t="s">
-        <v>91</v>
-      </c>
       <c r="E4" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F4" s="19"/>
     </row>
@@ -14433,31 +14431,31 @@
         <v>42</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D5" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="E5" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E5" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F5" s="19"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C6" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D6" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D6" s="21" t="s">
+      <c r="E6" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E6" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F6" s="19" t="s">
         <v>32</v>
@@ -14465,37 +14463,37 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="18" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C7" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D7" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D7" s="21" t="s">
+      <c r="E7" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E7" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F7" s="19"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="19" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C8" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D8" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D8" s="21" t="s">
+      <c r="E8" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E8" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F8" s="19"/>
     </row>
@@ -14507,31 +14505,31 @@
         <v>21</v>
       </c>
       <c r="C9" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="D9" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="D9" s="21" t="s">
-        <v>91</v>
-      </c>
       <c r="E9" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F9" s="19"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C10" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="D10" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="D10" s="21" t="s">
-        <v>91</v>
-      </c>
       <c r="E10" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F10" s="19"/>
     </row>
@@ -14543,31 +14541,31 @@
         <v>39</v>
       </c>
       <c r="C11" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="D11" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="D11" s="21" t="s">
-        <v>91</v>
-      </c>
       <c r="E11" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F11" s="19"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="19" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C12" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D12" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D12" s="21" t="s">
+      <c r="E12" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E12" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F12" s="19"/>
     </row>
@@ -14579,13 +14577,13 @@
         <v>31</v>
       </c>
       <c r="C13" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D13" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D13" s="21" t="s">
+      <c r="E13" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E13" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F13" s="19"/>
     </row>
@@ -14597,31 +14595,31 @@
         <v>28</v>
       </c>
       <c r="C14" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D14" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D14" s="21" t="s">
+      <c r="E14" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E14" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F14" s="19"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="18" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C15" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D15" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D15" s="21" t="s">
+      <c r="E15" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E15" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F15" s="19"/>
     </row>
@@ -14633,13 +14631,13 @@
         <v>37</v>
       </c>
       <c r="C16" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D16" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D16" s="21" t="s">
+      <c r="E16" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E16" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F16" s="19" t="s">
         <v>23</v>
@@ -14653,13 +14651,13 @@
         <v>52</v>
       </c>
       <c r="C17" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D17" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D17" s="21" t="s">
+      <c r="E17" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E17" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F17" s="19" t="s">
         <v>33</v>
@@ -14673,49 +14671,49 @@
         <v>33</v>
       </c>
       <c r="C18" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D18" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="E18" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E18" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F18" s="19"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="19" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C19" s="21" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D19" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="E19" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E19" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F19" s="19"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="19" t="s">
-        <v>58</v>
+        <v>95</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C20" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D20" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D20" s="21" t="s">
+      <c r="E20" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E20" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F20" s="19" t="s">
         <v>41</v>
@@ -14729,13 +14727,13 @@
         <v>57</v>
       </c>
       <c r="C21" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D21" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D21" s="21" t="s">
+      <c r="E21" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E21" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F21" s="19" t="s">
         <v>41</v>
@@ -14743,40 +14741,40 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="19" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C22" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D22" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D22" s="21" t="s">
+      <c r="E22" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E22" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F22" s="19"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="19" t="s">
+        <v>96</v>
+      </c>
+      <c r="B23" s="19" t="s">
+        <v>96</v>
+      </c>
+      <c r="C23" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D23" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="E23" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="F23" s="19" t="s">
         <v>97</v>
-      </c>
-      <c r="B23" s="19" t="s">
-        <v>97</v>
-      </c>
-      <c r="C23" s="21" t="s">
-        <v>87</v>
-      </c>
-      <c r="D23" s="21" t="s">
-        <v>88</v>
-      </c>
-      <c r="E23" s="21" t="s">
-        <v>89</v>
-      </c>
-      <c r="F23" s="19" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
@@ -14787,13 +14785,13 @@
         <v>43</v>
       </c>
       <c r="C24" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D24" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D24" s="21" t="s">
+      <c r="E24" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E24" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F24" s="19"/>
     </row>
@@ -14805,13 +14803,13 @@
         <v>51</v>
       </c>
       <c r="C25" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="D25" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="D25" s="21" t="s">
-        <v>91</v>
-      </c>
       <c r="E25" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F25" s="19" t="s">
         <v>49</v>
@@ -14825,13 +14823,13 @@
         <v>29</v>
       </c>
       <c r="C26" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="D26" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="D26" s="21" t="s">
-        <v>91</v>
-      </c>
       <c r="E26" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F26" s="19"/>
     </row>
@@ -14840,37 +14838,37 @@
         <v>38</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C27" s="21" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D27" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="E27" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E27" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F27" s="19"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C28" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="D28" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="D28" s="21" t="s">
-        <v>91</v>
-      </c>
       <c r="E28" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F28" s="19" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
@@ -14881,13 +14879,13 @@
         <v>35</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D29" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="E29" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E29" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F29" s="19"/>
     </row>
@@ -14899,13 +14897,13 @@
         <v>41</v>
       </c>
       <c r="C30" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="D30" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="D30" s="21" t="s">
-        <v>91</v>
-      </c>
       <c r="E30" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F30" s="19"/>
     </row>
@@ -14917,31 +14915,31 @@
         <v>47</v>
       </c>
       <c r="C31" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="D31" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="D31" s="21" t="s">
-        <v>91</v>
-      </c>
       <c r="E31" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F31" s="19"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B32" s="18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C32" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D32" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D32" s="21" t="s">
+      <c r="E32" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E32" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F32" s="19" t="s">
         <v>23</v>
@@ -14955,13 +14953,13 @@
         <v>49</v>
       </c>
       <c r="C33" s="21" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D33" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="E33" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E33" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F33" s="19"/>
     </row>
@@ -14973,13 +14971,13 @@
         <v>36</v>
       </c>
       <c r="C34" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D34" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D34" s="21" t="s">
+      <c r="E34" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E34" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F34" s="19"/>
     </row>
@@ -14991,16 +14989,16 @@
         <v>56</v>
       </c>
       <c r="C35" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="D35" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="D35" s="21" t="s">
-        <v>91</v>
-      </c>
       <c r="E35" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F35" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
@@ -15011,13 +15009,13 @@
         <v>32</v>
       </c>
       <c r="C36" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D36" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="E36" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E36" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F36" s="19"/>
     </row>
@@ -15029,13 +15027,13 @@
         <v>55</v>
       </c>
       <c r="C37" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="D37" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="D37" s="21" t="s">
-        <v>91</v>
-      </c>
       <c r="E37" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F37" s="19" t="s">
         <v>45</v>
@@ -15043,19 +15041,19 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="18" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B38" s="18" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C38" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D38" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D38" s="21" t="s">
+      <c r="E38" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E38" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F38" s="19"/>
     </row>
@@ -15064,16 +15062,16 @@
         <v>44</v>
       </c>
       <c r="B39" s="19" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D39" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="E39" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E39" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F39" s="19"/>
     </row>
@@ -15085,13 +15083,13 @@
         <v>50</v>
       </c>
       <c r="C40" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="D40" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="D40" s="21" t="s">
-        <v>91</v>
-      </c>
       <c r="E40" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F40" s="19" t="s">
         <v>49</v>
@@ -15099,19 +15097,19 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="19" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B41" s="19" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C41" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D41" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D41" s="21" t="s">
+      <c r="E41" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E41" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F41" s="19" t="s">
         <v>45</v>
@@ -15119,19 +15117,19 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="19" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B42" s="19" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C42" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D42" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D42" s="21" t="s">
+      <c r="E42" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E42" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F42" s="19"/>
     </row>
@@ -15143,31 +15141,31 @@
         <v>23</v>
       </c>
       <c r="C43" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="D43" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="D43" s="21" t="s">
-        <v>91</v>
-      </c>
       <c r="E43" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F43" s="19"/>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="18" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B44" s="18" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C44" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="D44" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="D44" s="21" t="s">
-        <v>91</v>
-      </c>
       <c r="E44" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F44" s="19"/>
     </row>
@@ -15179,31 +15177,31 @@
         <v>25</v>
       </c>
       <c r="C45" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D45" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D45" s="21" t="s">
+      <c r="E45" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E45" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F45" s="19"/>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="18" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B46" s="18" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C46" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D46" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D46" s="21" t="s">
+      <c r="E46" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E46" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F46" s="19" t="s">
         <v>26</v>
@@ -15217,51 +15215,51 @@
         <v>53</v>
       </c>
       <c r="C47" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D47" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D47" s="21" t="s">
+      <c r="E47" s="21" t="s">
         <v>88</v>
       </c>
-      <c r="E47" s="21" t="s">
-        <v>89</v>
-      </c>
       <c r="F47" s="19" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="19" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B48" s="19" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C48" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D48" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D48" s="21" t="s">
+      <c r="E48" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E48" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F48" s="19"/>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="19" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B49" s="19" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C49" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D49" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D49" s="21" t="s">
+      <c r="E49" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E49" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F49" s="19"/>
     </row>
@@ -15273,13 +15271,13 @@
         <v>26</v>
       </c>
       <c r="C50" s="21" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D50" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="E50" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E50" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F50" s="19"/>
     </row>
@@ -15291,13 +15289,13 @@
         <v>48</v>
       </c>
       <c r="C51" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D51" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D51" s="21" t="s">
+      <c r="E51" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E51" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F51" s="19"/>
     </row>
@@ -15309,31 +15307,31 @@
         <v>54</v>
       </c>
       <c r="C52" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="D52" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="D52" s="21" t="s">
-        <v>91</v>
-      </c>
       <c r="E52" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F52" s="19"/>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" s="18" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B53" s="18" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C53" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="D53" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="D53" s="21" t="s">
-        <v>91</v>
-      </c>
       <c r="E53" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F53" s="19"/>
     </row>
@@ -15345,13 +15343,13 @@
         <v>24</v>
       </c>
       <c r="C54" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D54" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D54" s="21" t="s">
+      <c r="E54" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E54" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F54" s="19"/>
     </row>
@@ -15363,13 +15361,13 @@
         <v>46</v>
       </c>
       <c r="C55" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="D55" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="D55" s="21" t="s">
-        <v>91</v>
-      </c>
       <c r="E55" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F55" s="19" t="s">
         <v>23</v>
@@ -15377,37 +15375,37 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" s="18" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B56" s="18" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C56" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D56" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D56" s="21" t="s">
+      <c r="E56" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E56" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F56" s="19"/>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" s="19" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B57" s="19" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C57" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="D57" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="D57" s="21" t="s">
-        <v>91</v>
-      </c>
       <c r="E57" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F57" s="19"/>
     </row>
@@ -15419,13 +15417,13 @@
         <v>40</v>
       </c>
       <c r="C58" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="D58" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="D58" s="21" t="s">
-        <v>91</v>
-      </c>
       <c r="E58" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F58" s="19" t="s">
         <v>33</v>
@@ -15439,13 +15437,13 @@
         <v>27</v>
       </c>
       <c r="C59" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D59" s="21" t="s">
+      <c r="E59" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E59" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F59" s="19"/>
     </row>
@@ -15457,31 +15455,31 @@
         <v>45</v>
       </c>
       <c r="C60" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D60" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D60" s="21" t="s">
+      <c r="E60" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E60" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F60" s="19"/>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" s="19" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B61" s="19" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C61" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="D61" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="D61" s="21" t="s">
-        <v>91</v>
-      </c>
       <c r="E61" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F61" s="19" t="s">
         <v>34</v>
@@ -15489,39 +15487,39 @@
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" s="19" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B62" s="19" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C62" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="D62" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="D62" s="21" t="s">
-        <v>91</v>
-      </c>
       <c r="E62" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F62" s="19" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" s="19" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B63" s="19" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C63" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D63" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D63" s="21" t="s">
+      <c r="E63" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E63" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F63" s="19"/>
     </row>
@@ -15533,49 +15531,49 @@
         <v>34</v>
       </c>
       <c r="C64" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D64" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D64" s="21" t="s">
+      <c r="E64" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E64" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F64" s="19"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" s="19" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B65" s="19" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C65" s="21" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D65" s="21" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E65" s="21" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F65" s="19"/>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" s="19" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B66" s="19" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C66" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D66" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="D66" s="21" t="s">
+      <c r="E66" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="E66" s="21" t="s">
-        <v>89</v>
       </c>
       <c r="F66" s="19"/>
     </row>
@@ -15598,37 +15596,37 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" s="15" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" s="15" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" s="15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" s="15" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" s="15" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" s="15" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>